<commit_message>
Added: Kapitel 4.6 bzw 4.7 Verkaufspreise in allen Modellen
Bilanznullpreise in die Modelle aufnehmen --> erledigt in FT, Methanol, Ammoniak
Bilanznullpreise bei Verkauf der Vorprodukte--> erledigt in FT, Methanol, Ammoniak
</commit_message>
<xml_diff>
--- a/Ammoniak/Ammoniak_Greenfield_Höchst/Datenbank.xlsx
+++ b/Ammoniak/Ammoniak_Greenfield_Höchst/Datenbank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak_Greenfield_Höchst\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak\Ammoniak_Greenfield_Höchst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8537F47-8298-4DE3-8ADF-36EF4CE0AC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8830D37-B7D8-4639-82CF-0991CC1903A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="299">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -1003,6 +1003,21 @@
   </si>
   <si>
     <t>Schattenvariable Einnahmen Stromverkauf</t>
+  </si>
+  <si>
+    <t>Verkaufspreiseanalyse</t>
+  </si>
+  <si>
+    <t>Maximaler Verkaufspreis Bilanznull</t>
+  </si>
+  <si>
+    <t>calc_maxprice</t>
+  </si>
+  <si>
+    <t>Verkaufspreis Bilanznull mit Vorverkauf</t>
+  </si>
+  <si>
+    <t>calc_price</t>
   </si>
 </sst>
 </file>
@@ -1265,49 +1280,49 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2562,7 +2577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" style="13" customWidth="1"/>
@@ -2595,10 +2610,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="78" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="75" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="29" t="s">
@@ -2613,8 +2628,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="73"/>
-      <c r="B3" s="75"/>
+      <c r="A3" s="80"/>
+      <c r="B3" s="73"/>
       <c r="C3" s="13" t="s">
         <v>136</v>
       </c>
@@ -2627,8 +2642,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="73"/>
-      <c r="B4" s="75"/>
+      <c r="A4" s="80"/>
+      <c r="B4" s="73"/>
       <c r="C4" s="13" t="s">
         <v>102</v>
       </c>
@@ -2641,8 +2656,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="73"/>
-      <c r="B5" s="75"/>
+      <c r="A5" s="80"/>
+      <c r="B5" s="73"/>
       <c r="C5" s="13" t="s">
         <v>172</v>
       </c>
@@ -2655,8 +2670,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="73"/>
-      <c r="B6" s="75"/>
+      <c r="A6" s="80"/>
+      <c r="B6" s="73"/>
       <c r="C6" s="13" t="s">
         <v>184</v>
       </c>
@@ -2669,8 +2684,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="73"/>
-      <c r="B7" s="75"/>
+      <c r="A7" s="80"/>
+      <c r="B7" s="73"/>
       <c r="C7" s="13" t="s">
         <v>202</v>
       </c>
@@ -2683,8 +2698,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="73"/>
-      <c r="B8" s="75"/>
+      <c r="A8" s="80"/>
+      <c r="B8" s="73"/>
       <c r="C8" s="13" t="s">
         <v>251</v>
       </c>
@@ -2697,8 +2712,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="73"/>
-      <c r="B9" s="75"/>
+      <c r="A9" s="80"/>
+      <c r="B9" s="73"/>
       <c r="C9" s="13" t="s">
         <v>216</v>
       </c>
@@ -2711,8 +2726,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="73"/>
-      <c r="B10" s="75"/>
+      <c r="A10" s="80"/>
+      <c r="B10" s="73"/>
       <c r="C10" s="13" t="s">
         <v>241</v>
       </c>
@@ -2725,13 +2740,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="73"/>
-      <c r="B11" s="75"/>
+      <c r="A11" s="80"/>
+      <c r="B11" s="73"/>
       <c r="E11" s="36"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="73"/>
-      <c r="B12" s="76" t="s">
+      <c r="A12" s="80"/>
+      <c r="B12" s="72" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="38" t="s">
@@ -2746,8 +2761,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="73"/>
-      <c r="B13" s="75"/>
+      <c r="A13" s="80"/>
+      <c r="B13" s="73"/>
       <c r="C13" s="13" t="s">
         <v>177</v>
       </c>
@@ -2760,8 +2775,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="73"/>
-      <c r="B14" s="75"/>
+      <c r="A14" s="80"/>
+      <c r="B14" s="73"/>
       <c r="C14" s="13" t="s">
         <v>180</v>
       </c>
@@ -2774,8 +2789,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="73"/>
-      <c r="B15" s="75"/>
+      <c r="A15" s="80"/>
+      <c r="B15" s="73"/>
       <c r="C15" s="13" t="s">
         <v>181</v>
       </c>
@@ -2788,8 +2803,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="73"/>
-      <c r="B16" s="75"/>
+      <c r="A16" s="80"/>
+      <c r="B16" s="73"/>
       <c r="C16" s="13" t="s">
         <v>102</v>
       </c>
@@ -2802,8 +2817,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="73"/>
-      <c r="B17" s="75"/>
+      <c r="A17" s="80"/>
+      <c r="B17" s="73"/>
       <c r="C17" s="13" t="s">
         <v>184</v>
       </c>
@@ -2816,8 +2831,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="73"/>
-      <c r="B18" s="75"/>
+      <c r="A18" s="80"/>
+      <c r="B18" s="73"/>
       <c r="C18" s="13" t="s">
         <v>202</v>
       </c>
@@ -2830,8 +2845,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="73"/>
-      <c r="B19" s="75"/>
+      <c r="A19" s="80"/>
+      <c r="B19" s="73"/>
       <c r="C19" s="13" t="s">
         <v>251</v>
       </c>
@@ -2844,8 +2859,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="73"/>
-      <c r="B20" s="75"/>
+      <c r="A20" s="80"/>
+      <c r="B20" s="73"/>
       <c r="C20" s="13" t="s">
         <v>216</v>
       </c>
@@ -2858,8 +2873,8 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="73"/>
-      <c r="B21" s="75"/>
+      <c r="A21" s="80"/>
+      <c r="B21" s="73"/>
       <c r="C21" s="13" t="s">
         <v>241</v>
       </c>
@@ -2872,16 +2887,16 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="73"/>
-      <c r="B22" s="77"/>
+      <c r="A22" s="80"/>
+      <c r="B22" s="76"/>
       <c r="C22" s="40"/>
       <c r="D22" s="40"/>
       <c r="E22" s="41"/>
       <c r="F22" s="40"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="73"/>
-      <c r="B23" s="78" t="s">
+      <c r="A23" s="80"/>
+      <c r="B23" s="83" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -2896,8 +2911,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="73"/>
-      <c r="B24" s="78"/>
+      <c r="A24" s="80"/>
+      <c r="B24" s="83"/>
       <c r="C24" s="13" t="s">
         <v>136</v>
       </c>
@@ -2910,8 +2925,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="73"/>
-      <c r="B25" s="78"/>
+      <c r="A25" s="80"/>
+      <c r="B25" s="83"/>
       <c r="C25" s="13" t="s">
         <v>102</v>
       </c>
@@ -2924,8 +2939,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="73"/>
-      <c r="B26" s="78"/>
+      <c r="A26" s="80"/>
+      <c r="B26" s="83"/>
       <c r="C26" s="13" t="s">
         <v>174</v>
       </c>
@@ -2938,8 +2953,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="73"/>
-      <c r="B27" s="78"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="83"/>
       <c r="C27" s="13" t="s">
         <v>184</v>
       </c>
@@ -2952,8 +2967,8 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="73"/>
-      <c r="B28" s="78"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="83"/>
       <c r="C28" s="13" t="s">
         <v>202</v>
       </c>
@@ -2966,8 +2981,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="73"/>
-      <c r="B29" s="78"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="83"/>
       <c r="C29" s="13" t="s">
         <v>251</v>
       </c>
@@ -2980,8 +2995,8 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="73"/>
-      <c r="B30" s="78"/>
+      <c r="A30" s="80"/>
+      <c r="B30" s="83"/>
       <c r="C30" s="13" t="s">
         <v>216</v>
       </c>
@@ -2994,8 +3009,8 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="73"/>
-      <c r="B31" s="78"/>
+      <c r="A31" s="80"/>
+      <c r="B31" s="83"/>
       <c r="C31" s="13" t="s">
         <v>241</v>
       </c>
@@ -3008,15 +3023,15 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="73"/>
-      <c r="B32" s="78"/>
+      <c r="A32" s="80"/>
+      <c r="B32" s="83"/>
       <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="72" t="s">
+      <c r="A33" s="78" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="80" t="s">
+      <c r="B33" s="86" t="s">
         <v>5</v>
       </c>
       <c r="C33" s="29" t="s">
@@ -3031,8 +3046,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="73"/>
-      <c r="B34" s="78"/>
+      <c r="A34" s="80"/>
+      <c r="B34" s="83"/>
       <c r="C34" s="13" t="s">
         <v>140</v>
       </c>
@@ -3045,8 +3060,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="73"/>
-      <c r="B35" s="78"/>
+      <c r="A35" s="80"/>
+      <c r="B35" s="83"/>
       <c r="C35" s="13" t="s">
         <v>169</v>
       </c>
@@ -3059,8 +3074,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="73"/>
-      <c r="B36" s="78"/>
+      <c r="A36" s="80"/>
+      <c r="B36" s="83"/>
       <c r="C36" s="13" t="s">
         <v>170</v>
       </c>
@@ -3073,8 +3088,8 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="73"/>
-      <c r="B37" s="78"/>
+      <c r="A37" s="80"/>
+      <c r="B37" s="83"/>
       <c r="C37" s="13" t="s">
         <v>184</v>
       </c>
@@ -3087,8 +3102,8 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="73"/>
-      <c r="B38" s="78"/>
+      <c r="A38" s="80"/>
+      <c r="B38" s="83"/>
       <c r="C38" s="13" t="s">
         <v>202</v>
       </c>
@@ -3101,8 +3116,8 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="73"/>
-      <c r="B39" s="78"/>
+      <c r="A39" s="80"/>
+      <c r="B39" s="83"/>
       <c r="C39" s="13" t="s">
         <v>251</v>
       </c>
@@ -3115,8 +3130,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="73"/>
-      <c r="B40" s="78"/>
+      <c r="A40" s="80"/>
+      <c r="B40" s="83"/>
       <c r="C40" s="13" t="s">
         <v>216</v>
       </c>
@@ -3129,8 +3144,8 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="73"/>
-      <c r="B41" s="78"/>
+      <c r="A41" s="80"/>
+      <c r="B41" s="83"/>
       <c r="C41" s="13" t="s">
         <v>241</v>
       </c>
@@ -3143,13 +3158,13 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="73"/>
-      <c r="B42" s="78"/>
+      <c r="A42" s="80"/>
+      <c r="B42" s="83"/>
       <c r="E42" s="36"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="73"/>
-      <c r="B43" s="81" t="s">
+      <c r="A43" s="80"/>
+      <c r="B43" s="82" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="38" t="s">
@@ -3164,8 +3179,8 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="73"/>
-      <c r="B44" s="78"/>
+      <c r="A44" s="80"/>
+      <c r="B44" s="83"/>
       <c r="C44" s="13" t="s">
         <v>142</v>
       </c>
@@ -3178,8 +3193,8 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="73"/>
-      <c r="B45" s="75"/>
+      <c r="A45" s="80"/>
+      <c r="B45" s="73"/>
       <c r="C45" s="13" t="s">
         <v>140</v>
       </c>
@@ -3192,8 +3207,8 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="73"/>
-      <c r="B46" s="75"/>
+      <c r="A46" s="80"/>
+      <c r="B46" s="73"/>
       <c r="C46" s="13" t="s">
         <v>136</v>
       </c>
@@ -3206,8 +3221,8 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="73"/>
-      <c r="B47" s="75"/>
+      <c r="A47" s="80"/>
+      <c r="B47" s="73"/>
       <c r="C47" s="13" t="s">
         <v>157</v>
       </c>
@@ -3220,8 +3235,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="73"/>
-      <c r="B48" s="75"/>
+      <c r="A48" s="80"/>
+      <c r="B48" s="73"/>
       <c r="C48" s="13" t="s">
         <v>158</v>
       </c>
@@ -3234,8 +3249,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="73"/>
-      <c r="B49" s="75"/>
+      <c r="A49" s="80"/>
+      <c r="B49" s="73"/>
       <c r="C49" s="13" t="s">
         <v>184</v>
       </c>
@@ -3248,8 +3263,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="73"/>
-      <c r="B50" s="75"/>
+      <c r="A50" s="80"/>
+      <c r="B50" s="73"/>
       <c r="C50" s="13" t="s">
         <v>202</v>
       </c>
@@ -3262,8 +3277,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="73"/>
-      <c r="B51" s="75"/>
+      <c r="A51" s="80"/>
+      <c r="B51" s="73"/>
       <c r="C51" s="13" t="s">
         <v>251</v>
       </c>
@@ -3276,8 +3291,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="73"/>
-      <c r="B52" s="75"/>
+      <c r="A52" s="80"/>
+      <c r="B52" s="73"/>
       <c r="C52" s="13" t="s">
         <v>216</v>
       </c>
@@ -3290,8 +3305,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="73"/>
-      <c r="B53" s="75"/>
+      <c r="A53" s="80"/>
+      <c r="B53" s="73"/>
       <c r="C53" s="13" t="s">
         <v>241</v>
       </c>
@@ -3304,18 +3319,18 @@
       </c>
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="79"/>
-      <c r="B54" s="82"/>
+      <c r="A54" s="81"/>
+      <c r="B54" s="74"/>
       <c r="C54" s="44"/>
       <c r="D54" s="44"/>
       <c r="E54" s="45"/>
       <c r="F54" s="44"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="72" t="s">
+      <c r="A55" s="78" t="s">
         <v>86</v>
       </c>
-      <c r="B55" s="74" t="s">
+      <c r="B55" s="75" t="s">
         <v>87</v>
       </c>
       <c r="C55" s="29" t="s">
@@ -3330,8 +3345,8 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="73"/>
-      <c r="B56" s="75"/>
+      <c r="A56" s="80"/>
+      <c r="B56" s="73"/>
       <c r="C56" s="13" t="s">
         <v>200</v>
       </c>
@@ -3344,13 +3359,13 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="73"/>
-      <c r="B57" s="77"/>
+      <c r="A57" s="80"/>
+      <c r="B57" s="76"/>
       <c r="E57" s="34"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="73"/>
-      <c r="B58" s="81" t="s">
+      <c r="A58" s="80"/>
+      <c r="B58" s="82" t="s">
         <v>6</v>
       </c>
       <c r="C58" s="38" t="s">
@@ -3365,8 +3380,8 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="73"/>
-      <c r="B59" s="78"/>
+      <c r="A59" s="80"/>
+      <c r="B59" s="83"/>
       <c r="C59" s="13" t="s">
         <v>136</v>
       </c>
@@ -3379,8 +3394,8 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="73"/>
-      <c r="B60" s="78"/>
+      <c r="A60" s="80"/>
+      <c r="B60" s="83"/>
       <c r="C60" s="13" t="s">
         <v>152</v>
       </c>
@@ -3393,8 +3408,8 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="73"/>
-      <c r="B61" s="78"/>
+      <c r="A61" s="80"/>
+      <c r="B61" s="83"/>
       <c r="C61" s="13" t="s">
         <v>184</v>
       </c>
@@ -3407,8 +3422,8 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="73"/>
-      <c r="B62" s="78"/>
+      <c r="A62" s="80"/>
+      <c r="B62" s="83"/>
       <c r="C62" s="13" t="s">
         <v>202</v>
       </c>
@@ -3421,8 +3436,8 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="73"/>
-      <c r="B63" s="78"/>
+      <c r="A63" s="80"/>
+      <c r="B63" s="83"/>
       <c r="C63" s="13" t="s">
         <v>210</v>
       </c>
@@ -3435,8 +3450,8 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="73"/>
-      <c r="B64" s="78"/>
+      <c r="A64" s="80"/>
+      <c r="B64" s="83"/>
       <c r="C64" s="13" t="s">
         <v>251</v>
       </c>
@@ -3449,8 +3464,8 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="73"/>
-      <c r="B65" s="78"/>
+      <c r="A65" s="80"/>
+      <c r="B65" s="83"/>
       <c r="C65" s="13" t="s">
         <v>216</v>
       </c>
@@ -3463,8 +3478,8 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="73"/>
-      <c r="B66" s="78"/>
+      <c r="A66" s="80"/>
+      <c r="B66" s="83"/>
       <c r="C66" s="13" t="s">
         <v>241</v>
       </c>
@@ -3477,12 +3492,12 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="73"/>
-      <c r="B67" s="85"/>
+      <c r="A67" s="80"/>
+      <c r="B67" s="84"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="73"/>
-      <c r="B68" s="81" t="s">
+      <c r="A68" s="80"/>
+      <c r="B68" s="82" t="s">
         <v>7</v>
       </c>
       <c r="C68" s="38" t="s">
@@ -3497,8 +3512,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="73"/>
-      <c r="B69" s="78"/>
+      <c r="A69" s="80"/>
+      <c r="B69" s="83"/>
       <c r="C69" s="13" t="s">
         <v>137</v>
       </c>
@@ -3511,8 +3526,8 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="73"/>
-      <c r="B70" s="78"/>
+      <c r="A70" s="80"/>
+      <c r="B70" s="83"/>
       <c r="C70" s="13" t="s">
         <v>150</v>
       </c>
@@ -3525,8 +3540,8 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="73"/>
-      <c r="B71" s="78"/>
+      <c r="A71" s="80"/>
+      <c r="B71" s="83"/>
       <c r="C71" s="13" t="s">
         <v>184</v>
       </c>
@@ -3539,8 +3554,8 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="73"/>
-      <c r="B72" s="78"/>
+      <c r="A72" s="80"/>
+      <c r="B72" s="83"/>
       <c r="C72" s="13" t="s">
         <v>202</v>
       </c>
@@ -3553,8 +3568,8 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="73"/>
-      <c r="B73" s="78"/>
+      <c r="A73" s="80"/>
+      <c r="B73" s="83"/>
       <c r="C73" s="13" t="s">
         <v>210</v>
       </c>
@@ -3567,8 +3582,8 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="73"/>
-      <c r="B74" s="78"/>
+      <c r="A74" s="80"/>
+      <c r="B74" s="83"/>
       <c r="C74" s="13" t="s">
         <v>251</v>
       </c>
@@ -3581,8 +3596,8 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="73"/>
-      <c r="B75" s="78"/>
+      <c r="A75" s="80"/>
+      <c r="B75" s="83"/>
       <c r="C75" s="13" t="s">
         <v>216</v>
       </c>
@@ -3595,8 +3610,8 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="73"/>
-      <c r="B76" s="78"/>
+      <c r="A76" s="80"/>
+      <c r="B76" s="83"/>
       <c r="C76" s="13" t="s">
         <v>241</v>
       </c>
@@ -3609,14 +3624,14 @@
       </c>
     </row>
     <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="79"/>
-      <c r="B77" s="86"/>
+      <c r="A77" s="81"/>
+      <c r="B77" s="85"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="72" t="s">
+      <c r="A78" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="B78" s="74" t="s">
+      <c r="B78" s="75" t="s">
         <v>87</v>
       </c>
       <c r="C78" s="29" t="s">
@@ -3631,8 +3646,8 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="84"/>
-      <c r="B79" s="83"/>
+      <c r="A79" s="79"/>
+      <c r="B79" s="77"/>
       <c r="C79" s="56" t="s">
         <v>293</v>
       </c>
@@ -3645,8 +3660,8 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="73"/>
-      <c r="B80" s="75"/>
+      <c r="A80" s="80"/>
+      <c r="B80" s="73"/>
       <c r="C80" s="13" t="s">
         <v>196</v>
       </c>
@@ -3659,13 +3674,13 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="73"/>
-      <c r="B81" s="77"/>
+      <c r="A81" s="80"/>
+      <c r="B81" s="76"/>
       <c r="E81" s="36"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="73"/>
-      <c r="B82" s="76" t="s">
+      <c r="A82" s="80"/>
+      <c r="B82" s="72" t="s">
         <v>93</v>
       </c>
       <c r="C82" s="38" t="s">
@@ -3680,8 +3695,8 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="73"/>
-      <c r="B83" s="75"/>
+      <c r="A83" s="80"/>
+      <c r="B83" s="73"/>
       <c r="C83" s="13" t="s">
         <v>197</v>
       </c>
@@ -3694,16 +3709,16 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="73"/>
-      <c r="B84" s="77"/>
+      <c r="A84" s="80"/>
+      <c r="B84" s="76"/>
       <c r="C84" s="40"/>
       <c r="D84" s="40"/>
       <c r="E84" s="41"/>
       <c r="F84" s="40"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="73"/>
-      <c r="B85" s="76" t="s">
+      <c r="A85" s="80"/>
+      <c r="B85" s="72" t="s">
         <v>94</v>
       </c>
       <c r="C85" s="13" t="s">
@@ -3718,8 +3733,8 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="73"/>
-      <c r="B86" s="75"/>
+      <c r="A86" s="80"/>
+      <c r="B86" s="73"/>
       <c r="C86" s="13" t="s">
         <v>198</v>
       </c>
@@ -3732,18 +3747,18 @@
       </c>
     </row>
     <row r="87" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="79"/>
-      <c r="B87" s="82"/>
+      <c r="A87" s="81"/>
+      <c r="B87" s="74"/>
       <c r="C87" s="44"/>
       <c r="D87" s="44"/>
       <c r="E87" s="45"/>
       <c r="F87" s="44"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="72" t="s">
+      <c r="A88" s="78" t="s">
         <v>212</v>
       </c>
-      <c r="B88" s="74" t="s">
+      <c r="B88" s="75" t="s">
         <v>15</v>
       </c>
       <c r="C88" s="29" t="s">
@@ -3758,8 +3773,8 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="84"/>
-      <c r="B89" s="75"/>
+      <c r="A89" s="79"/>
+      <c r="B89" s="73"/>
       <c r="C89" s="13" t="s">
         <v>225</v>
       </c>
@@ -3771,16 +3786,16 @@
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="84"/>
-      <c r="B90" s="77"/>
+      <c r="A90" s="79"/>
+      <c r="B90" s="76"/>
       <c r="C90" s="40"/>
       <c r="D90" s="40"/>
       <c r="E90" s="40"/>
       <c r="F90" s="40"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="84"/>
-      <c r="B91" s="76" t="s">
+      <c r="A91" s="79"/>
+      <c r="B91" s="72" t="s">
         <v>235</v>
       </c>
       <c r="C91" s="13" t="s">
@@ -3794,8 +3809,8 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="84"/>
-      <c r="B92" s="75"/>
+      <c r="A92" s="79"/>
+      <c r="B92" s="73"/>
       <c r="C92" s="13" t="s">
         <v>233</v>
       </c>
@@ -3807,8 +3822,8 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="84"/>
-      <c r="B93" s="75"/>
+      <c r="A93" s="79"/>
+      <c r="B93" s="73"/>
       <c r="C93" s="13" t="s">
         <v>229</v>
       </c>
@@ -3820,8 +3835,8 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="84"/>
-      <c r="B94" s="75"/>
+      <c r="A94" s="79"/>
+      <c r="B94" s="73"/>
       <c r="C94" s="13" t="s">
         <v>231</v>
       </c>
@@ -3833,8 +3848,8 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="84"/>
-      <c r="B95" s="75"/>
+      <c r="A95" s="79"/>
+      <c r="B95" s="73"/>
       <c r="C95" s="13" t="s">
         <v>234</v>
       </c>
@@ -3846,8 +3861,8 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="84"/>
-      <c r="B96" s="75"/>
+      <c r="A96" s="79"/>
+      <c r="B96" s="73"/>
       <c r="C96" s="13" t="s">
         <v>244</v>
       </c>
@@ -3859,8 +3874,8 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="84"/>
-      <c r="B97" s="76" t="s">
+      <c r="A97" s="79"/>
+      <c r="B97" s="72" t="s">
         <v>265</v>
       </c>
       <c r="C97" s="38" t="s">
@@ -3875,8 +3890,8 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="84"/>
-      <c r="B98" s="83"/>
+      <c r="A98" s="79"/>
+      <c r="B98" s="77"/>
       <c r="C98" s="56" t="s">
         <v>261</v>
       </c>
@@ -3889,8 +3904,8 @@
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="84"/>
-      <c r="B99" s="83"/>
+      <c r="A99" s="79"/>
+      <c r="B99" s="77"/>
       <c r="C99" s="56" t="s">
         <v>276</v>
       </c>
@@ -3903,8 +3918,8 @@
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="84"/>
-      <c r="B100" s="83"/>
+      <c r="A100" s="79"/>
+      <c r="B100" s="77"/>
       <c r="C100" s="56" t="s">
         <v>262</v>
       </c>
@@ -3917,8 +3932,8 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="84"/>
-      <c r="B101" s="83"/>
+      <c r="A101" s="79"/>
+      <c r="B101" s="77"/>
       <c r="C101" s="56" t="s">
         <v>278</v>
       </c>
@@ -3931,8 +3946,8 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="84"/>
-      <c r="B102" s="83"/>
+      <c r="A102" s="79"/>
+      <c r="B102" s="77"/>
       <c r="C102" s="56" t="s">
         <v>282</v>
       </c>
@@ -3945,8 +3960,8 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="84"/>
-      <c r="B103" s="83"/>
+      <c r="A103" s="79"/>
+      <c r="B103" s="77"/>
       <c r="C103" s="56" t="s">
         <v>259</v>
       </c>
@@ -3959,8 +3974,8 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="84"/>
-      <c r="B104" s="83"/>
+      <c r="A104" s="79"/>
+      <c r="B104" s="77"/>
       <c r="C104" s="56" t="s">
         <v>263</v>
       </c>
@@ -3973,8 +3988,8 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="84"/>
-      <c r="B105" s="83"/>
+      <c r="A105" s="79"/>
+      <c r="B105" s="77"/>
       <c r="C105" s="56" t="s">
         <v>264</v>
       </c>
@@ -3987,8 +4002,8 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="84"/>
-      <c r="B106" s="76" t="s">
+      <c r="A106" s="79"/>
+      <c r="B106" s="72" t="s">
         <v>283</v>
       </c>
       <c r="C106" s="38" t="s">
@@ -4003,8 +4018,8 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="84"/>
-      <c r="B107" s="83"/>
+      <c r="A107" s="79"/>
+      <c r="B107" s="77"/>
       <c r="C107" s="56" t="s">
         <v>286</v>
       </c>
@@ -4017,8 +4032,8 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="84"/>
-      <c r="B108" s="83"/>
+      <c r="A108" s="79"/>
+      <c r="B108" s="77"/>
       <c r="C108" s="56" t="s">
         <v>288</v>
       </c>
@@ -4031,8 +4046,8 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="84"/>
-      <c r="B109" s="83"/>
+      <c r="A109" s="79"/>
+      <c r="B109" s="77"/>
       <c r="C109" s="13" t="s">
         <v>289</v>
       </c>
@@ -4043,13 +4058,57 @@
         <v>274</v>
       </c>
     </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="79"/>
+      <c r="B110" s="76"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="79"/>
+      <c r="B111" s="72" t="s">
+        <v>294</v>
+      </c>
+      <c r="C111" s="38" t="s">
+        <v>295</v>
+      </c>
+      <c r="D111" s="38" t="s">
+        <v>296</v>
+      </c>
+      <c r="E111" s="38"/>
+      <c r="F111" s="38" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="79"/>
+      <c r="B112" s="73"/>
+      <c r="C112" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="D112" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="F112" s="13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="79"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="B106:B110"/>
+    <mergeCell ref="A88:A113"/>
+    <mergeCell ref="A2:A32"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="A33:A54"/>
+    <mergeCell ref="B33:B42"/>
+    <mergeCell ref="B43:B54"/>
     <mergeCell ref="B85:B87"/>
     <mergeCell ref="B55:B57"/>
     <mergeCell ref="B91:B96"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="A88:A109"/>
     <mergeCell ref="B97:B105"/>
     <mergeCell ref="B88:B90"/>
     <mergeCell ref="A55:A77"/>
@@ -4058,13 +4117,6 @@
     <mergeCell ref="A78:A87"/>
     <mergeCell ref="B78:B81"/>
     <mergeCell ref="B82:B84"/>
-    <mergeCell ref="A2:A32"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="B23:B32"/>
-    <mergeCell ref="A33:A54"/>
-    <mergeCell ref="B33:B42"/>
-    <mergeCell ref="B43:B54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>